<commit_message>
Añadiendo nueva categoria a la historia
</commit_message>
<xml_diff>
--- a/scripts/libreria.xlsx
+++ b/scripts/libreria.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Superusuario\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Superusuario\Documents\dashboard-rodenstock\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADF4CAA-E677-4D4F-8154-C6B39915B15C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D70E8C-2DA1-488A-92D5-1CFD2067700D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="90">
   <si>
     <t>Categoria</t>
   </si>
@@ -298,13 +298,16 @@
   </si>
   <si>
     <t xml:space="preserve">SV organic </t>
+  </si>
+  <si>
+    <t>Single Vision 1.60</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,6 +334,20 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -386,7 +403,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -403,6 +420,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -893,7 +916,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I113"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -1752,7 +1775,7 @@
       </c>
       <c r="D64" s="1"/>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:6">
       <c r="A65" s="1" t="s">
         <v>50</v>
       </c>
@@ -1764,7 +1787,7 @@
       </c>
       <c r="D65" s="1"/>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:6">
       <c r="A66" s="1" t="s">
         <v>50</v>
       </c>
@@ -1776,7 +1799,7 @@
       </c>
       <c r="D66" s="1"/>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:6">
       <c r="A67" s="1" t="s">
         <v>50</v>
       </c>
@@ -1788,7 +1811,7 @@
       </c>
       <c r="D67" s="1"/>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:6">
       <c r="A68" s="1" t="s">
         <v>50</v>
       </c>
@@ -1800,7 +1823,7 @@
       </c>
       <c r="D68" s="1"/>
     </row>
-    <row r="69" spans="1:4" ht="25.5">
+    <row r="69" spans="1:6" ht="25.5">
       <c r="A69" s="1" t="s">
         <v>50</v>
       </c>
@@ -1812,7 +1835,7 @@
       </c>
       <c r="D69" s="1"/>
     </row>
-    <row r="70" spans="1:4">
+    <row r="70" spans="1:6">
       <c r="A70" s="1" t="s">
         <v>50</v>
       </c>
@@ -1824,7 +1847,7 @@
       </c>
       <c r="D70" s="1"/>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:6">
       <c r="A71" s="1" t="s">
         <v>50</v>
       </c>
@@ -1836,7 +1859,7 @@
       </c>
       <c r="D71" s="1"/>
     </row>
-    <row r="72" spans="1:4">
+    <row r="72" spans="1:6">
       <c r="A72" s="1" t="s">
         <v>50</v>
       </c>
@@ -1850,7 +1873,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" spans="1:6">
       <c r="A73" s="1" t="s">
         <v>50</v>
       </c>
@@ -1864,7 +1887,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:6">
       <c r="A74" s="1" t="s">
         <v>50</v>
       </c>
@@ -1878,7 +1901,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:6">
       <c r="A75" s="1" t="s">
         <v>50</v>
       </c>
@@ -1892,7 +1915,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:6">
       <c r="A76" s="1" t="s">
         <v>50</v>
       </c>
@@ -1906,7 +1929,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="25.5">
+    <row r="77" spans="1:6" ht="26.25" thickBot="1">
       <c r="A77" s="1" t="s">
         <v>50</v>
       </c>
@@ -1917,64 +1940,65 @@
         <v>73</v>
       </c>
       <c r="D77" s="1"/>
-    </row>
-    <row r="78" spans="1:4">
+      <c r="F77" s="7"/>
+    </row>
+    <row r="78" spans="1:6" ht="15.75" thickBot="1">
       <c r="A78" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C78" s="1" t="s">
-        <v>58</v>
+      <c r="C78" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="15.75" thickBot="1">
       <c r="A79" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C79" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="15.75" thickBot="1">
+      <c r="A80" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4">
-      <c r="A80" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:6">
       <c r="A81" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:6">
       <c r="A82" s="1" t="s">
         <v>50</v>
       </c>
@@ -1982,13 +2006,13 @@
         <v>72</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:6">
       <c r="A83" s="1" t="s">
         <v>50</v>
       </c>
@@ -1996,82 +2020,81 @@
         <v>72</v>
       </c>
       <c r="C83" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D83" s="1"/>
-    </row>
-    <row r="84" spans="1:7">
-      <c r="A84" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D84" s="1"/>
-    </row>
-    <row r="85" spans="1:7">
+      <c r="D84" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
       <c r="A85" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="F85" s="2"/>
-    </row>
-    <row r="86" spans="1:7">
+        <v>72</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D85" s="1"/>
+    </row>
+    <row r="86" spans="1:6">
       <c r="A86" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C86" s="4" t="s">
+      <c r="C86" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D86" s="1"/>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C87" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F86" s="2"/>
-    </row>
-    <row r="87" spans="1:7">
-      <c r="A87" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F87" s="3"/>
-    </row>
-    <row r="88" spans="1:7">
+      <c r="F87" s="2"/>
+    </row>
+    <row r="88" spans="1:6">
       <c r="A88" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="89" spans="1:7">
+      <c r="F88" s="2"/>
+    </row>
+    <row r="89" spans="1:6">
       <c r="A89" s="1" t="s">
         <v>50</v>
       </c>
@@ -2079,13 +2102,14 @@
         <v>72</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7">
+        <v>74</v>
+      </c>
+      <c r="F89" s="3"/>
+    </row>
+    <row r="90" spans="1:6">
       <c r="A90" s="1" t="s">
         <v>50</v>
       </c>
@@ -2093,13 +2117,13 @@
         <v>72</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:6">
       <c r="A91" s="1" t="s">
         <v>50</v>
       </c>
@@ -2107,51 +2131,53 @@
         <v>72</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:6">
       <c r="A92" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C92" s="1"/>
+        <v>72</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>54</v>
+      </c>
       <c r="D92" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
       <c r="A93" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D93" s="1"/>
-    </row>
-    <row r="94" spans="1:7">
+        <v>55</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
       <c r="A94" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C94" s="1" t="s">
-        <v>81</v>
-      </c>
+      <c r="C94" s="1"/>
       <c r="D94" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
       <c r="A95" s="1" t="s">
         <v>50</v>
       </c>
@@ -2159,13 +2185,11 @@
         <v>26</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D95" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="96" spans="1:7">
+      <c r="D95" s="1"/>
+    </row>
+    <row r="96" spans="1:6">
       <c r="A96" s="1" t="s">
         <v>50</v>
       </c>
@@ -2176,10 +2200,8 @@
         <v>81</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F96" s="3"/>
-      <c r="G96" s="3"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="1" t="s">
@@ -2189,9 +2211,11 @@
         <v>26</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D97" s="1"/>
+        <v>82</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="1" t="s">
@@ -2201,9 +2225,13 @@
         <v>26</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D98" s="1"/>
+        <v>81</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="1" t="s">
@@ -2212,57 +2240,82 @@
       <c r="B99" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C99" s="1"/>
-      <c r="D99" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="C99" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D99" s="1"/>
     </row>
     <row r="100" spans="1:9">
       <c r="A100" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C100" s="1"/>
-      <c r="D100" s="1" t="s">
-        <v>85</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D100" s="1"/>
     </row>
     <row r="101" spans="1:9">
       <c r="A101" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B101" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C101" s="1"/>
+      <c r="D101" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9">
+      <c r="A102" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B102" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C101" t="s">
+      <c r="C102" s="1"/>
+      <c r="D102" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9">
+      <c r="A103" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C103" t="s">
         <v>86</v>
       </c>
-      <c r="D101" s="1" t="s">
+      <c r="D103" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
-      <c r="A102" s="1"/>
-      <c r="B102" s="1"/>
-    </row>
-    <row r="108" spans="1:9">
-      <c r="I108" s="3"/>
+    <row r="104" spans="1:9">
+      <c r="A104" s="1"/>
+      <c r="B104" s="1"/>
     </row>
     <row r="110" spans="1:9">
-      <c r="H110" s="5"/>
-    </row>
-    <row r="111" spans="1:9">
-      <c r="H111" s="5"/>
+      <c r="I110" s="3"/>
     </row>
     <row r="112" spans="1:9">
       <c r="H112" s="5"/>
     </row>
     <row r="113" spans="8:8">
-      <c r="H113" s="3"/>
+      <c r="H113" s="5"/>
+    </row>
+    <row r="114" spans="8:8">
+      <c r="H114" s="5"/>
+    </row>
+    <row r="115" spans="8:8">
+      <c r="H115" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Streamlit theme config
</commit_message>
<xml_diff>
--- a/scripts/libreria.xlsx
+++ b/scripts/libreria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Superusuario\Documents\dashboard-rodenstock\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D70E8C-2DA1-488A-92D5-1CFD2067700D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B35E5BF8-9463-4DB5-9BEA-43D438D04BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -307,7 +307,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -319,36 +319,29 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="10"/>
       <color rgb="FF202124"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.5"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <u/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -359,42 +352,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF0C67DF"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF0C67DF"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF0C67DF"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF0C67DF"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -403,29 +366,26 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -917,12 +877,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I115"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="21" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22" style="2" customWidth="1"/>
+    <col min="3" max="3" width="36.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -988,7 +949,7 @@
       <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -1114,7 +1075,7 @@
       <c r="B14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1156,7 +1117,7 @@
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -1267,7 +1228,7 @@
       <c r="B26" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="1"/>
@@ -1345,7 +1306,7 @@
       <c r="B32" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -1471,7 +1432,7 @@
       <c r="B41" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D41" s="1" t="s">
@@ -1513,7 +1474,7 @@
       <c r="B44" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D44" s="1" t="s">
@@ -1624,7 +1585,7 @@
       <c r="B53" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D53" s="1"/>
@@ -1702,9 +1663,9 @@
       <c r="D59" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F59" s="2"/>
-      <c r="G59" s="2"/>
-      <c r="H59" s="2"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="1" t="s">
@@ -1717,9 +1678,9 @@
         <v>54</v>
       </c>
       <c r="D60" s="1"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="1" t="s">
@@ -1732,9 +1693,9 @@
         <v>55</v>
       </c>
       <c r="D61" s="1"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="2"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="1" t="s">
@@ -1929,7 +1890,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="26.25" thickBot="1">
+    <row r="77" spans="1:6" ht="25.5">
       <c r="A77" s="1" t="s">
         <v>50</v>
       </c>
@@ -1940,37 +1901,37 @@
         <v>73</v>
       </c>
       <c r="D77" s="1"/>
-      <c r="F77" s="7"/>
-    </row>
-    <row r="78" spans="1:6" ht="15.75" thickBot="1">
+      <c r="F77" s="4"/>
+    </row>
+    <row r="78" spans="1:6">
       <c r="A78" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C78" s="6" t="s">
+      <c r="C78" s="5" t="s">
         <v>89</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="15.75" thickBot="1">
+    <row r="79" spans="1:6">
       <c r="A79" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C79" s="6" t="s">
+      <c r="C79" s="5" t="s">
         <v>89</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="15.75" thickBot="1">
+    <row r="80" spans="1:6">
       <c r="A80" s="1" t="s">
         <v>50</v>
       </c>
@@ -2071,13 +2032,13 @@
       <c r="B87" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C87" s="4" t="s">
+      <c r="C87" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F87" s="2"/>
+      <c r="F87" s="3"/>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="1" t="s">
@@ -2086,13 +2047,13 @@
       <c r="B88" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C88" s="4" t="s">
+      <c r="C88" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F88" s="2"/>
+      <c r="F88" s="3"/>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="1" t="s">
@@ -2288,7 +2249,7 @@
       <c r="B103" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C103" t="s">
+      <c r="C103" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D103" s="1" t="s">
@@ -2303,13 +2264,13 @@
       <c r="I110" s="3"/>
     </row>
     <row r="112" spans="1:9">
-      <c r="H112" s="5"/>
+      <c r="H112" s="6"/>
     </row>
     <row r="113" spans="8:8">
-      <c r="H113" s="5"/>
+      <c r="H113" s="6"/>
     </row>
     <row r="114" spans="8:8">
-      <c r="H114" s="5"/>
+      <c r="H114" s="6"/>
     </row>
     <row r="115" spans="8:8">
       <c r="H115" s="3"/>

</xml_diff>